<commit_message>
latest commit of code and data
</commit_message>
<xml_diff>
--- a/src/tree_measurements_code/PICOS_ADAIR_manual_root_crown_analysis_ANOVA_tables.xlsx
+++ b/src/tree_measurements_code/PICOS_ADAIR_manual_root_crown_analysis_ANOVA_tables.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25712"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <xr:revisionPtr revIDLastSave="0" documentId="11_713058713D77B485E3D15741E4B29A0072049BAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
@@ -13,8 +13,22 @@
     <sheet name="PICOS_Root_mixed_models" sheetId="3" r:id="rId3"/>
     <sheet name="ADAIR_Root_mixed_models" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>

</xml_diff>